<commit_message>
Add print setup to the transport/export workbooks
Landscape A4, fit-to-width, repeated header row on every page, and
tighter margins for the tabular sheets; portrait for the memo-style
sheets (重要品目メモ, 該非判定書_手順). Makes both workbooks usable as
printed handouts without columns getting cut off or headers
disappearing after page 1.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U9UL7uC3hEPvevtvxay711
</commit_message>
<xml_diff>
--- a/Equipments/Transport_to_Aachen/DACNV_Equipment_List_輸送分類.xlsx
+++ b/Equipments/Transport_to_Aachen/DACNV_Equipment_List_輸送分類.xlsx
@@ -13,7 +13,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'機材一覧'!$A$4:$E$57</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'機材一覧'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'輸送分類'!$A$4:$N$57</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'輸送分類'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
@@ -870,7 +872,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5" customHeight="1"/>
@@ -2478,7 +2480,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:E57"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="0"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;P / &amp;N ページ&amp;R&amp;D</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -2486,7 +2498,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -6063,7 +6075,17 @@
   <mergeCells count="1">
     <mergeCell ref="A2:L2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="0"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;P / &amp;N ページ&amp;R&amp;D</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -6071,7 +6093,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -8186,7 +8208,17 @@
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="0"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;P / &amp;N ページ&amp;R&amp;D</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -8194,7 +8226,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -8400,6 +8432,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="0"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;P / &amp;N ページ&amp;R&amp;D</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>